<commit_message>
Analyse und Diagramme abgeschlossen
</commit_message>
<xml_diff>
--- a/excel/Praxisnachbereitung-SS25.xlsx
+++ b/excel/Praxisnachbereitung-SS25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noelrabenschlag/Desktop/praxisnachbereitung-ss25/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9DFBEF3-EE31-E341-A052-7B5DB0777244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101D802C-8FBC-3F4F-B24E-B0E433CE2671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="220" yWindow="660" windowWidth="29400" windowHeight="16760" activeTab="3" xr2:uid="{6A8FE1CE-64E8-0943-B336-CBBA9009EA98}"/>
   </bookViews>
@@ -16,15 +16,19 @@
     <sheet name="Ausleihen" sheetId="7" r:id="rId1"/>
     <sheet name="Geraete" sheetId="3" r:id="rId2"/>
     <sheet name="Mitarbeiter" sheetId="4" r:id="rId3"/>
-    <sheet name="Gesamt" sheetId="8" r:id="rId4"/>
+    <sheet name="PivotTable" sheetId="9" r:id="rId4"/>
+    <sheet name="Gesamt" sheetId="8" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">Ausleihen!$A$1:$D$46</definedName>
     <definedName name="ExterneDaten_1" localSheetId="1" hidden="1">Geraete!$A$1:$F$36</definedName>
-    <definedName name="ExterneDaten_1" localSheetId="3" hidden="1">Gesamt!$A$1:$D$46</definedName>
+    <definedName name="ExterneDaten_1" localSheetId="4" hidden="1">Gesamt!$A$1:$D$46</definedName>
     <definedName name="ExterneDaten_1" localSheetId="2" hidden="1">Mitarbeiter!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="4" r:id="rId6"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -68,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="103">
   <si>
     <t>Gerätenummer</t>
   </si>
@@ -365,6 +369,18 @@
   </si>
   <si>
     <t>Standort2</t>
+  </si>
+  <si>
+    <t>Zeilenbeschriftungen</t>
+  </si>
+  <si>
+    <t>Gesamtergebnis</t>
+  </si>
+  <si>
+    <t>Anzahl von Gerätenummer</t>
+  </si>
+  <si>
+    <t>Spaltenbeschriftungen</t>
   </si>
 </sst>
 </file>
@@ -374,10 +390,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -427,10 +449,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -439,11 +462,52 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="38">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -535,6 +599,2062 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Praxisnachbereitung-SS25.xlsx]PivotTable!PivotTable1</c:name>
+    <c:fmtId val="1"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>PivotTable!$B$3:$B$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Berlin</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>PivotTable!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Beamer</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Drucker</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Smartphone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Tablet</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>PivotTable!$B$5:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A743-824C-A37F-ABBAB25EFBD3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>PivotTable!$C$3:$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Hamburg</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>PivotTable!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Beamer</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Drucker</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Smartphone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Tablet</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>PivotTable!$C$5:$C$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-A743-824C-A37F-ABBAB25EFBD3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>PivotTable!$D$3:$D$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>München</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>PivotTable!$A$5:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Beamer</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Drucker</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Smartphone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Tablet</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>PivotTable!$D$5:$D$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-A743-824C-A37F-ABBAB25EFBD3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="100"/>
+        <c:axId val="390013247"/>
+        <c:axId val="767058687"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="390013247"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="767058687"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="767058687"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="390013247"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Diagramm 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94A9BCF2-58A2-21BB-AFB3-E5E6D227D8CE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Noel Rabenschlag" refreshedDate="46102.604774652777" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="45" xr:uid="{412A981F-D7B5-6348-8050-2037B1DBC46D}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Ausleihen__32"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Gerätenummer" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Mitarbeiter-ID" numFmtId="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1001" maxValue="1012"/>
+    </cacheField>
+    <cacheField name="Ausgabe am" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2023-12-01T00:00:00" maxDate="2025-10-01T00:00:00"/>
+    </cacheField>
+    <cacheField name="Rückgabe am" numFmtId="14">
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2024-06-27T00:00:00" maxDate="2025-10-06T00:00:00"/>
+    </cacheField>
+    <cacheField name="Gerätetyp" numFmtId="0">
+      <sharedItems count="6">
+        <s v="Beamer"/>
+        <s v="Monitor"/>
+        <s v="Drucker"/>
+        <s v="Smartphone"/>
+        <s v="Laptop"/>
+        <s v="Tablet"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Modell" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Kaufdatum" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2021-03-03T00:00:00" maxDate="2025-09-10T00:00:00"/>
+    </cacheField>
+    <cacheField name="Netto-Kaufpreis" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="141.71" maxValue="1898.65"/>
+    </cacheField>
+    <cacheField name="Standort" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Berlin"/>
+        <s v="München"/>
+        <s v="Hamburg"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Name" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Abteilung" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Standort2" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="45">
+  <r>
+    <s v="G0035"/>
+    <n v="1009"/>
+    <d v="2024-05-09T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="BenQ MW550"/>
+    <d v="2024-01-03T00:00:00"/>
+    <n v="644.54"/>
+    <x v="0"/>
+    <s v="Univ.Prof. Heimo Karge"/>
+    <s v="Marketing"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0021"/>
+    <n v="1008"/>
+    <d v="2025-09-30T00:00:00"/>
+    <d v="2025-10-05T00:00:00"/>
+    <x v="1"/>
+    <s v="Samsung Curved"/>
+    <d v="2023-02-22T00:00:00"/>
+    <n v="1134.1600000000001"/>
+    <x v="1"/>
+    <s v="Dipl.-Ing. Klaus-Werner Holsten B.Sc."/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0024"/>
+    <n v="1005"/>
+    <d v="2025-03-27T00:00:00"/>
+    <d v="2025-07-30T00:00:00"/>
+    <x v="1"/>
+    <s v="Dell UltraSharp"/>
+    <d v="2022-03-01T00:00:00"/>
+    <n v="750.91"/>
+    <x v="0"/>
+    <s v="Alexandre Davids"/>
+    <s v="Vertrieb"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0016"/>
+    <n v="1010"/>
+    <d v="2025-07-28T00:00:00"/>
+    <m/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2023-03-30T00:00:00"/>
+    <n v="1501.06"/>
+    <x v="0"/>
+    <s v="Carolin Hande"/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0006"/>
+    <n v="1012"/>
+    <d v="2025-05-31T00:00:00"/>
+    <d v="2025-06-10T00:00:00"/>
+    <x v="3"/>
+    <s v="Samsung S21"/>
+    <d v="2024-01-01T00:00:00"/>
+    <n v="1257.96"/>
+    <x v="1"/>
+    <s v="Ariane Klemt-Kaul"/>
+    <s v="IT"/>
+    <s v="München"/>
+  </r>
+  <r>
+    <s v="G0005"/>
+    <n v="1009"/>
+    <d v="2024-04-07T00:00:00"/>
+    <m/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2021-11-03T00:00:00"/>
+    <n v="823.23"/>
+    <x v="0"/>
+    <s v="Univ.Prof. Heimo Karge"/>
+    <s v="Marketing"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0009"/>
+    <n v="1011"/>
+    <d v="2025-07-12T00:00:00"/>
+    <d v="2025-07-15T00:00:00"/>
+    <x v="4"/>
+    <s v="Dell XPS"/>
+    <d v="2023-04-10T00:00:00"/>
+    <n v="1458.02"/>
+    <x v="1"/>
+    <s v="Auguste Davids"/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0011"/>
+    <n v="1005"/>
+    <d v="2025-06-29T00:00:00"/>
+    <d v="2025-08-29T00:00:00"/>
+    <x v="2"/>
+    <s v="Brother HL"/>
+    <d v="2025-09-09T00:00:00"/>
+    <n v="141.71"/>
+    <x v="1"/>
+    <s v="Alexandre Davids"/>
+    <s v="Vertrieb"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0028"/>
+    <n v="1004"/>
+    <d v="2024-08-19T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="Epson EB"/>
+    <d v="2023-01-19T00:00:00"/>
+    <n v="1246.58"/>
+    <x v="2"/>
+    <s v="Klemens Löffler"/>
+    <s v="Vertrieb"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0013"/>
+    <n v="1012"/>
+    <d v="2024-05-07T00:00:00"/>
+    <d v="2024-06-27T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2021-05-16T00:00:00"/>
+    <n v="1898.65"/>
+    <x v="2"/>
+    <s v="Ariane Klemt-Kaul"/>
+    <s v="IT"/>
+    <s v="München"/>
+  </r>
+  <r>
+    <s v="G0024"/>
+    <n v="1008"/>
+    <d v="2024-03-24T00:00:00"/>
+    <m/>
+    <x v="1"/>
+    <s v="Dell UltraSharp"/>
+    <d v="2022-03-01T00:00:00"/>
+    <n v="750.91"/>
+    <x v="0"/>
+    <s v="Dipl.-Ing. Klaus-Werner Holsten B.Sc."/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0029"/>
+    <n v="1002"/>
+    <d v="2025-09-21T00:00:00"/>
+    <d v="2025-10-04T00:00:00"/>
+    <x v="4"/>
+    <s v="Lenovo ThinkPad"/>
+    <d v="2021-05-21T00:00:00"/>
+    <n v="1553.15"/>
+    <x v="2"/>
+    <s v="Eleni Hauffer"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0005"/>
+    <n v="1006"/>
+    <d v="2025-08-23T00:00:00"/>
+    <d v="2025-09-22T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2021-11-03T00:00:00"/>
+    <n v="823.23"/>
+    <x v="0"/>
+    <s v="Eric Patberg B.Sc."/>
+    <s v="Vertrieb"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0015"/>
+    <n v="1010"/>
+    <d v="2024-03-26T00:00:00"/>
+    <d v="2025-08-17T00:00:00"/>
+    <x v="3"/>
+    <s v="iPhone 13"/>
+    <d v="2022-09-20T00:00:00"/>
+    <n v="661.44"/>
+    <x v="1"/>
+    <s v="Carolin Hande"/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0005"/>
+    <n v="1012"/>
+    <d v="2024-11-03T00:00:00"/>
+    <m/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2021-11-03T00:00:00"/>
+    <n v="823.23"/>
+    <x v="0"/>
+    <s v="Ariane Klemt-Kaul"/>
+    <s v="IT"/>
+    <s v="München"/>
+  </r>
+  <r>
+    <s v="G0015"/>
+    <n v="1002"/>
+    <d v="2024-08-15T00:00:00"/>
+    <m/>
+    <x v="3"/>
+    <s v="iPhone 13"/>
+    <d v="2022-09-20T00:00:00"/>
+    <n v="661.44"/>
+    <x v="1"/>
+    <s v="Eleni Hauffer"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0022"/>
+    <n v="1002"/>
+    <d v="2025-08-30T00:00:00"/>
+    <d v="2025-09-30T00:00:00"/>
+    <x v="5"/>
+    <s v="iPad"/>
+    <d v="2024-08-20T00:00:00"/>
+    <n v="1591.98"/>
+    <x v="2"/>
+    <s v="Eleni Hauffer"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0018"/>
+    <n v="1011"/>
+    <d v="2024-10-03T00:00:00"/>
+    <d v="2024-11-27T00:00:00"/>
+    <x v="5"/>
+    <s v="iPad"/>
+    <d v="2022-10-05T00:00:00"/>
+    <n v="1688.07"/>
+    <x v="1"/>
+    <s v="Auguste Davids"/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0035"/>
+    <n v="1003"/>
+    <d v="2024-05-05T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="BenQ MW550"/>
+    <d v="2024-01-03T00:00:00"/>
+    <n v="644.54"/>
+    <x v="0"/>
+    <s v="Paul Dobes-Stiffel"/>
+    <s v="Produktion"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0031"/>
+    <n v="1004"/>
+    <d v="2024-01-29T00:00:00"/>
+    <m/>
+    <x v="4"/>
+    <s v="HP EliteBook"/>
+    <d v="2025-04-28T00:00:00"/>
+    <n v="1095.6199999999999"/>
+    <x v="1"/>
+    <s v="Klemens Löffler"/>
+    <s v="Vertrieb"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0027"/>
+    <n v="1004"/>
+    <d v="2024-04-21T00:00:00"/>
+    <d v="2025-07-01T00:00:00"/>
+    <x v="1"/>
+    <s v="Samsung Curved"/>
+    <d v="2022-07-24T00:00:00"/>
+    <n v="501.64"/>
+    <x v="1"/>
+    <s v="Klemens Löffler"/>
+    <s v="Vertrieb"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0028"/>
+    <n v="1006"/>
+    <d v="2024-12-04T00:00:00"/>
+    <d v="2025-03-16T00:00:00"/>
+    <x v="0"/>
+    <s v="Epson EB"/>
+    <d v="2023-01-19T00:00:00"/>
+    <n v="1246.58"/>
+    <x v="2"/>
+    <s v="Eric Patberg B.Sc."/>
+    <s v="Vertrieb"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0030"/>
+    <n v="1012"/>
+    <d v="2025-05-15T00:00:00"/>
+    <d v="2025-09-05T00:00:00"/>
+    <x v="0"/>
+    <s v="Epson EB"/>
+    <d v="2022-03-27T00:00:00"/>
+    <n v="1629.76"/>
+    <x v="1"/>
+    <s v="Ariane Klemt-Kaul"/>
+    <s v="IT"/>
+    <s v="München"/>
+  </r>
+  <r>
+    <s v="G0007"/>
+    <n v="1001"/>
+    <d v="2024-09-09T00:00:00"/>
+    <d v="2025-07-16T00:00:00"/>
+    <x v="4"/>
+    <s v="Lenovo ThinkPad"/>
+    <d v="2021-06-13T00:00:00"/>
+    <n v="869.09"/>
+    <x v="2"/>
+    <s v="Aleksandr Weinhage"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0022"/>
+    <n v="1002"/>
+    <d v="2024-07-20T00:00:00"/>
+    <d v="2025-01-06T00:00:00"/>
+    <x v="5"/>
+    <s v="iPad"/>
+    <d v="2024-08-20T00:00:00"/>
+    <n v="1591.98"/>
+    <x v="2"/>
+    <s v="Eleni Hauffer"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0013"/>
+    <n v="1009"/>
+    <d v="2024-01-28T00:00:00"/>
+    <d v="2025-02-26T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2021-05-16T00:00:00"/>
+    <n v="1898.65"/>
+    <x v="2"/>
+    <s v="Univ.Prof. Heimo Karge"/>
+    <s v="Marketing"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0028"/>
+    <n v="1003"/>
+    <d v="2024-10-30T00:00:00"/>
+    <d v="2024-12-04T00:00:00"/>
+    <x v="0"/>
+    <s v="Epson EB"/>
+    <d v="2023-01-19T00:00:00"/>
+    <n v="1246.58"/>
+    <x v="2"/>
+    <s v="Paul Dobes-Stiffel"/>
+    <s v="Produktion"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0016"/>
+    <n v="1002"/>
+    <d v="2025-05-22T00:00:00"/>
+    <d v="2025-05-31T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2023-03-30T00:00:00"/>
+    <n v="1501.06"/>
+    <x v="0"/>
+    <s v="Eleni Hauffer"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0007"/>
+    <n v="1001"/>
+    <d v="2025-08-11T00:00:00"/>
+    <m/>
+    <x v="4"/>
+    <s v="Lenovo ThinkPad"/>
+    <d v="2021-06-13T00:00:00"/>
+    <n v="869.09"/>
+    <x v="2"/>
+    <s v="Aleksandr Weinhage"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0035"/>
+    <n v="1001"/>
+    <d v="2024-01-06T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="BenQ MW550"/>
+    <d v="2024-01-03T00:00:00"/>
+    <n v="644.54"/>
+    <x v="0"/>
+    <s v="Aleksandr Weinhage"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0016"/>
+    <n v="1003"/>
+    <d v="2024-02-08T00:00:00"/>
+    <d v="2025-06-09T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2023-03-30T00:00:00"/>
+    <n v="1501.06"/>
+    <x v="0"/>
+    <s v="Paul Dobes-Stiffel"/>
+    <s v="Produktion"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0031"/>
+    <n v="1004"/>
+    <d v="2024-02-14T00:00:00"/>
+    <m/>
+    <x v="4"/>
+    <s v="HP EliteBook"/>
+    <d v="2025-04-28T00:00:00"/>
+    <n v="1095.6199999999999"/>
+    <x v="1"/>
+    <s v="Klemens Löffler"/>
+    <s v="Vertrieb"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0004"/>
+    <n v="1003"/>
+    <d v="2025-06-19T00:00:00"/>
+    <d v="2025-09-08T00:00:00"/>
+    <x v="4"/>
+    <s v="Dell XPS"/>
+    <d v="2025-05-05T00:00:00"/>
+    <n v="1007.88"/>
+    <x v="1"/>
+    <s v="Paul Dobes-Stiffel"/>
+    <s v="Produktion"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0025"/>
+    <n v="1005"/>
+    <d v="2025-01-18T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="Epson EB"/>
+    <d v="2023-12-06T00:00:00"/>
+    <n v="545.46"/>
+    <x v="0"/>
+    <s v="Alexandre Davids"/>
+    <s v="Vertrieb"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0030"/>
+    <n v="1005"/>
+    <d v="2023-12-01T00:00:00"/>
+    <d v="2024-09-24T00:00:00"/>
+    <x v="0"/>
+    <s v="Epson EB"/>
+    <d v="2022-03-27T00:00:00"/>
+    <n v="1629.76"/>
+    <x v="1"/>
+    <s v="Alexandre Davids"/>
+    <s v="Vertrieb"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0032"/>
+    <n v="1003"/>
+    <d v="2024-08-04T00:00:00"/>
+    <d v="2025-08-02T00:00:00"/>
+    <x v="4"/>
+    <s v="Lenovo ThinkPad"/>
+    <d v="2022-11-11T00:00:00"/>
+    <n v="1801.36"/>
+    <x v="1"/>
+    <s v="Paul Dobes-Stiffel"/>
+    <s v="Produktion"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0014"/>
+    <n v="1001"/>
+    <d v="2024-11-26T00:00:00"/>
+    <d v="2025-03-03T00:00:00"/>
+    <x v="4"/>
+    <s v="Lenovo ThinkPad"/>
+    <d v="2021-03-03T00:00:00"/>
+    <n v="1415.97"/>
+    <x v="2"/>
+    <s v="Aleksandr Weinhage"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0035"/>
+    <n v="1001"/>
+    <d v="2024-12-15T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="BenQ MW550"/>
+    <d v="2024-01-03T00:00:00"/>
+    <n v="644.54"/>
+    <x v="0"/>
+    <s v="Aleksandr Weinhage"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0004"/>
+    <n v="1001"/>
+    <d v="2025-08-11T00:00:00"/>
+    <d v="2025-08-12T00:00:00"/>
+    <x v="4"/>
+    <s v="Dell XPS"/>
+    <d v="2025-05-05T00:00:00"/>
+    <n v="1007.88"/>
+    <x v="1"/>
+    <s v="Aleksandr Weinhage"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0033"/>
+    <n v="1009"/>
+    <d v="2025-03-24T00:00:00"/>
+    <d v="2025-05-07T00:00:00"/>
+    <x v="0"/>
+    <s v="BenQ MW550"/>
+    <d v="2022-03-03T00:00:00"/>
+    <n v="1212.29"/>
+    <x v="0"/>
+    <s v="Univ.Prof. Heimo Karge"/>
+    <s v="Marketing"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0033"/>
+    <n v="1002"/>
+    <d v="2025-03-25T00:00:00"/>
+    <m/>
+    <x v="0"/>
+    <s v="BenQ MW550"/>
+    <d v="2022-03-03T00:00:00"/>
+    <n v="1212.29"/>
+    <x v="0"/>
+    <s v="Eleni Hauffer"/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0005"/>
+    <n v="1010"/>
+    <d v="2025-08-30T00:00:00"/>
+    <d v="2025-09-25T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2021-11-03T00:00:00"/>
+    <n v="823.23"/>
+    <x v="0"/>
+    <s v="Carolin Hande"/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0016"/>
+    <n v="1007"/>
+    <d v="2025-05-18T00:00:00"/>
+    <d v="2025-07-08T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2023-03-30T00:00:00"/>
+    <n v="1501.06"/>
+    <x v="0"/>
+    <s v="Orhan Siering MBA."/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+  <r>
+    <s v="G0016"/>
+    <n v="1010"/>
+    <d v="2025-05-31T00:00:00"/>
+    <d v="2025-10-02T00:00:00"/>
+    <x v="2"/>
+    <s v="Canon Pixma"/>
+    <d v="2023-03-30T00:00:00"/>
+    <n v="1501.06"/>
+    <x v="0"/>
+    <s v="Carolin Hande"/>
+    <s v="IT"/>
+    <s v="Hamburg"/>
+  </r>
+  <r>
+    <s v="G0006"/>
+    <n v="1007"/>
+    <d v="2024-07-03T00:00:00"/>
+    <m/>
+    <x v="3"/>
+    <s v="Samsung S21"/>
+    <d v="2024-01-01T00:00:00"/>
+    <n v="1257.96"/>
+    <x v="1"/>
+    <s v="Orhan Siering MBA."/>
+    <s v="IT"/>
+    <s v="Berlin"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E349C4E0-5D9B-2C42-9626-F4963B86E8BA}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+  <location ref="A3:E11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="8"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Anzahl von Gerätenummer" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="1" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="1" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExterneDaten_1" connectionId="3" xr16:uid="{D1B75854-CCA3-F545-804F-356AD4BC2914}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="5">
@@ -601,10 +2721,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{85309FFA-F8FC-F24F-AB57-53C2C883CE11}" name="Ausleihen__3" displayName="Ausleihen__3" ref="A1:D46" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D46" xr:uid="{85309FFA-F8FC-F24F-AB57-53C2C883CE11}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{68D34859-38B7-B84D-9513-C75817798680}" uniqueName="1" name="Gerätenummer" queryTableFieldId="1" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{08F50FDD-7B92-A244-B0FA-790F7F9F537F}" uniqueName="2" name="Mitarbeiter-ID" queryTableFieldId="2" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{68302F70-7F17-DF44-B3C3-5F634AFC18B9}" uniqueName="3" name="Ausgabe am" queryTableFieldId="3" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{F7E3878C-611A-3942-BB13-6D97F90C6756}" uniqueName="4" name="Rückgabe am" queryTableFieldId="4" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{68D34859-38B7-B84D-9513-C75817798680}" uniqueName="1" name="Gerätenummer" queryTableFieldId="1" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{08F50FDD-7B92-A244-B0FA-790F7F9F537F}" uniqueName="2" name="Mitarbeiter-ID" queryTableFieldId="2" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{68302F70-7F17-DF44-B3C3-5F634AFC18B9}" uniqueName="3" name="Ausgabe am" queryTableFieldId="3" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{F7E3878C-611A-3942-BB13-6D97F90C6756}" uniqueName="4" name="Rückgabe am" queryTableFieldId="4" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -614,12 +2734,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{592EA434-AABE-1A4D-982F-E0E1287E1467}" name="Geraete" displayName="Geraete" ref="A1:F36" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F36" xr:uid="{592EA434-AABE-1A4D-982F-E0E1287E1467}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{15493AA0-5BF0-A545-90B3-9414C47EC1F2}" uniqueName="1" name="Gerätenummer" queryTableFieldId="1" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{D4A7CBDA-F02B-8144-A922-D4B8E5323845}" uniqueName="2" name="Gerätetyp" queryTableFieldId="2" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{2973C530-E2AE-104F-9359-A67D6FF31844}" uniqueName="3" name="Modell" queryTableFieldId="3" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{456DF500-324B-C346-B5CF-0AA159CFB2AA}" uniqueName="4" name="Kaufdatum" queryTableFieldId="4" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{0466FA76-F957-7B41-B81E-4E055DC3E455}" uniqueName="5" name="Netto-Kaufpreis" queryTableFieldId="5" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{1AD5D242-50BD-A344-AC3A-9A57AB7F8D3D}" uniqueName="6" name="Standort" queryTableFieldId="6" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{15493AA0-5BF0-A545-90B3-9414C47EC1F2}" uniqueName="1" name="Gerätenummer" queryTableFieldId="1" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{D4A7CBDA-F02B-8144-A922-D4B8E5323845}" uniqueName="2" name="Gerätetyp" queryTableFieldId="2" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{2973C530-E2AE-104F-9359-A67D6FF31844}" uniqueName="3" name="Modell" queryTableFieldId="3" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{456DF500-324B-C346-B5CF-0AA159CFB2AA}" uniqueName="4" name="Kaufdatum" queryTableFieldId="4" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{0466FA76-F957-7B41-B81E-4E055DC3E455}" uniqueName="5" name="Netto-Kaufpreis" queryTableFieldId="5" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{1AD5D242-50BD-A344-AC3A-9A57AB7F8D3D}" uniqueName="6" name="Standort" queryTableFieldId="6" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -629,45 +2749,44 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7894F2B9-D7EF-5D4C-AD4A-66D61A0D5C22}" name="Mitarbeiter" displayName="Mitarbeiter" ref="A1:D13" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D13" xr:uid="{7894F2B9-D7EF-5D4C-AD4A-66D61A0D5C22}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{82419368-56EF-E043-8052-5B199CD342E3}" uniqueName="1" name="Mitarbeiter-ID" queryTableFieldId="1" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{E5C3136C-90A5-A14C-AFC8-F6E383C0E333}" uniqueName="2" name="Name" queryTableFieldId="2" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{788A5330-106B-2D44-A36B-AA8592E48732}" uniqueName="3" name="Abteilung" queryTableFieldId="3" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{1E52BF6D-5D62-7E48-BF68-A81CCBE37FDB}" uniqueName="4" name="Standort" queryTableFieldId="4" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{82419368-56EF-E043-8052-5B199CD342E3}" uniqueName="1" name="Mitarbeiter-ID" queryTableFieldId="1" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{E5C3136C-90A5-A14C-AFC8-F6E383C0E333}" uniqueName="2" name="Name" queryTableFieldId="2" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{788A5330-106B-2D44-A36B-AA8592E48732}" uniqueName="3" name="Abteilung" queryTableFieldId="3" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{1E52BF6D-5D62-7E48-BF68-A81CCBE37FDB}" uniqueName="4" name="Standort" queryTableFieldId="4" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{698FB23A-8A57-2A47-93ED-9044A3110072}" name="Ausleihen__32" displayName="Ausleihen__32" ref="A1:L46" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:L46" xr:uid="{698FB23A-8A57-2A47-93ED-9044A3110072}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{698FB23A-8A57-2A47-93ED-9044A3110072}" name="Ausleihen__32" displayName="Ausleihen__32" ref="A1:L47" tableType="queryTable" totalsRowCount="1">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{AA34A09F-F420-C74C-9CF3-2AD6DE9A6A15}" uniqueName="1" name="Gerätenummer" queryTableFieldId="1" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{CCA91D1B-480B-0E4E-A03A-5E107BCF4BE6}" uniqueName="2" name="Mitarbeiter-ID" queryTableFieldId="2" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{C8FFFFA7-181A-AF49-8302-2EBDC2AE5BEB}" uniqueName="3" name="Ausgabe am" queryTableFieldId="3" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{1F10113B-CD1F-214D-A328-9E01EA8C9AEF}" uniqueName="4" name="Rückgabe am" queryTableFieldId="4" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{3B4CAB0E-45AC-C148-9E96-BF26B7821015}" uniqueName="5" name="Gerätetyp" queryTableFieldId="5" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{AA34A09F-F420-C74C-9CF3-2AD6DE9A6A15}" uniqueName="1" name="Gerätenummer" queryTableFieldId="1" dataDxfId="23" totalsRowDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{CCA91D1B-480B-0E4E-A03A-5E107BCF4BE6}" uniqueName="2" name="Mitarbeiter-ID" queryTableFieldId="2" dataDxfId="22" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{C8FFFFA7-181A-AF49-8302-2EBDC2AE5BEB}" uniqueName="3" name="Ausgabe am" queryTableFieldId="3" dataDxfId="21" totalsRowDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{1F10113B-CD1F-214D-A328-9E01EA8C9AEF}" uniqueName="4" name="Rückgabe am" queryTableFieldId="4" dataDxfId="20" totalsRowDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{3B4CAB0E-45AC-C148-9E96-BF26B7821015}" uniqueName="5" name="Gerätetyp" queryTableFieldId="5" dataDxfId="19" totalsRowDxfId="7">
       <calculatedColumnFormula>VLOOKUP(A2,Geraete!A:F,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{1F413BB6-3601-2542-A191-43F09B591E6B}" uniqueName="6" name="Modell" queryTableFieldId="6" dataDxfId="6">
+    <tableColumn id="6" xr3:uid="{1F413BB6-3601-2542-A191-43F09B591E6B}" uniqueName="6" name="Modell" queryTableFieldId="6" dataDxfId="18" totalsRowDxfId="6">
       <calculatedColumnFormula>VLOOKUP(A2,Geraete!A:F,3,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{E4AFFEA0-4311-5A44-880E-51D1DEE65E94}" uniqueName="7" name="Kaufdatum" queryTableFieldId="7" dataDxfId="5">
+    <tableColumn id="7" xr3:uid="{E4AFFEA0-4311-5A44-880E-51D1DEE65E94}" uniqueName="7" name="Kaufdatum" queryTableFieldId="7" dataDxfId="17" totalsRowDxfId="5">
       <calculatedColumnFormula>VLOOKUP(A2,Geraete!A:F,4,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{16C14272-0C12-8243-AA84-4490F978BFE0}" uniqueName="8" name="Netto-Kaufpreis" queryTableFieldId="8" dataDxfId="4">
+    <tableColumn id="8" xr3:uid="{16C14272-0C12-8243-AA84-4490F978BFE0}" uniqueName="8" name="Netto-Kaufpreis" queryTableFieldId="8" dataDxfId="16" totalsRowDxfId="4">
       <calculatedColumnFormula>VLOOKUP(A2,Geraete!A:F,5,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{E7B2B921-538A-574B-AB32-61A891D59516}" uniqueName="9" name="Standort" queryTableFieldId="9" dataDxfId="3">
+    <tableColumn id="9" xr3:uid="{E7B2B921-538A-574B-AB32-61A891D59516}" uniqueName="9" name="Standort" queryTableFieldId="9" dataDxfId="15" totalsRowDxfId="3">
       <calculatedColumnFormula>VLOOKUP(A2,Geraete!A:F,6,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{2311476C-EF1C-7D45-BC18-C30DD7E704C5}" uniqueName="11" name="Name" queryTableFieldId="11" dataDxfId="2">
+    <tableColumn id="11" xr3:uid="{2311476C-EF1C-7D45-BC18-C30DD7E704C5}" uniqueName="11" name="Name" queryTableFieldId="11" dataDxfId="14" totalsRowDxfId="2">
       <calculatedColumnFormula>VLOOKUP(B2&amp;"",Mitarbeiter!$A:$D,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{9DC0D57F-C912-F046-A6A2-C7A5C72C9EBF}" uniqueName="12" name="Abteilung" queryTableFieldId="12" dataDxfId="1">
+    <tableColumn id="12" xr3:uid="{9DC0D57F-C912-F046-A6A2-C7A5C72C9EBF}" uniqueName="12" name="Abteilung" queryTableFieldId="12" dataDxfId="13" totalsRowDxfId="1">
       <calculatedColumnFormula>VLOOKUP(B2&amp;"",Mitarbeiter!$A:$D,3,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1F79EB2D-9D4D-8C4F-B88C-0244B71614AF}" uniqueName="13" name="Standort2" queryTableFieldId="13" dataDxfId="0">
+    <tableColumn id="13" xr3:uid="{1F79EB2D-9D4D-8C4F-B88C-0244B71614AF}" uniqueName="13" name="Standort2" queryTableFieldId="13" dataDxfId="12" totalsRowDxfId="0">
       <calculatedColumnFormula>VLOOKUP(B2&amp;"",Mitarbeiter!$A:$D,4,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -996,7 +3115,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
   </cols>
@@ -1005,7 +3124,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1016,10 +3135,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="9">
         <v>1009</v>
       </c>
       <c r="C2" s="1">
@@ -1030,7 +3149,7 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>1008</v>
       </c>
       <c r="C3" s="1">
@@ -1044,7 +3163,7 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>1005</v>
       </c>
       <c r="C4" s="1">
@@ -1058,7 +3177,7 @@
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <v>1010</v>
       </c>
       <c r="C5" s="1">
@@ -1069,7 +3188,7 @@
       <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>1012</v>
       </c>
       <c r="C6" s="1">
@@ -1083,7 +3202,7 @@
       <c r="A7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <v>1009</v>
       </c>
       <c r="C7" s="1">
@@ -1094,7 +3213,7 @@
       <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="9">
         <v>1011</v>
       </c>
       <c r="C8" s="1">
@@ -1108,7 +3227,7 @@
       <c r="A9" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="9">
         <v>1005</v>
       </c>
       <c r="C9" s="1">
@@ -1122,7 +3241,7 @@
       <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <v>1004</v>
       </c>
       <c r="C10" s="1">
@@ -1133,7 +3252,7 @@
       <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <v>1012</v>
       </c>
       <c r="C11" s="1">
@@ -1147,7 +3266,7 @@
       <c r="A12" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <v>1008</v>
       </c>
       <c r="C12" s="1">
@@ -1158,7 +3277,7 @@
       <c r="A13" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>1002</v>
       </c>
       <c r="C13" s="1">
@@ -1172,7 +3291,7 @@
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>1006</v>
       </c>
       <c r="C14" s="1">
@@ -1186,7 +3305,7 @@
       <c r="A15" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="9">
         <v>1010</v>
       </c>
       <c r="C15" s="1">
@@ -1195,13 +3314,13 @@
       <c r="D15" s="1">
         <v>45886</v>
       </c>
-      <c r="F15" s="4"/>
+      <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="9">
         <v>1012</v>
       </c>
       <c r="C16" s="1">
@@ -1212,7 +3331,7 @@
       <c r="A17" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="9">
         <v>1002</v>
       </c>
       <c r="C17" s="1">
@@ -1223,7 +3342,7 @@
       <c r="A18" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>1002</v>
       </c>
       <c r="C18" s="1">
@@ -1237,7 +3356,7 @@
       <c r="A19" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>1011</v>
       </c>
       <c r="C19" s="1">
@@ -1248,10 +3367,10 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>1003</v>
       </c>
       <c r="C20" s="1">
@@ -1262,7 +3381,7 @@
       <c r="A21" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="9">
         <v>1004</v>
       </c>
       <c r="C21" s="1">
@@ -1273,7 +3392,7 @@
       <c r="A22" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="9">
         <v>1004</v>
       </c>
       <c r="C22" s="1">
@@ -1287,7 +3406,7 @@
       <c r="A23" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="9">
         <v>1006</v>
       </c>
       <c r="C23" s="1">
@@ -1301,7 +3420,7 @@
       <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="9">
         <v>1012</v>
       </c>
       <c r="C24" s="1">
@@ -1315,7 +3434,7 @@
       <c r="A25" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="9">
         <v>1001</v>
       </c>
       <c r="C25" s="1">
@@ -1329,7 +3448,7 @@
       <c r="A26" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>1002</v>
       </c>
       <c r="C26" s="1">
@@ -1343,7 +3462,7 @@
       <c r="A27" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>1009</v>
       </c>
       <c r="C27" s="1">
@@ -1357,7 +3476,7 @@
       <c r="A28" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="9">
         <v>1003</v>
       </c>
       <c r="C28" s="1">
@@ -1368,10 +3487,10 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>1002</v>
       </c>
       <c r="C29" s="1">
@@ -1385,7 +3504,7 @@
       <c r="A30" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="9">
         <v>1001</v>
       </c>
       <c r="C30" s="1">
@@ -1396,7 +3515,7 @@
       <c r="A31" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="9">
         <v>1001</v>
       </c>
       <c r="C31" s="1">
@@ -1404,10 +3523,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="9">
         <v>1003</v>
       </c>
       <c r="C32" s="1">
@@ -1421,7 +3540,7 @@
       <c r="A33" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="9">
         <v>1004</v>
       </c>
       <c r="C33" s="1">
@@ -1429,10 +3548,10 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="9">
         <v>1003</v>
       </c>
       <c r="C34" s="1">
@@ -1446,7 +3565,7 @@
       <c r="A35" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="9">
         <v>1005</v>
       </c>
       <c r="C35" s="1">
@@ -1457,7 +3576,7 @@
       <c r="A36" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="9">
         <v>1005</v>
       </c>
       <c r="C36" s="1">
@@ -1471,7 +3590,7 @@
       <c r="A37" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>1003</v>
       </c>
       <c r="C37" s="1">
@@ -1485,7 +3604,7 @@
       <c r="A38" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>1001</v>
       </c>
       <c r="C38" s="1">
@@ -1496,10 +3615,10 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="9" t="s">
+      <c r="A39" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="9">
         <v>1001</v>
       </c>
       <c r="C39" s="1">
@@ -1507,10 +3626,10 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B40" s="8">
+      <c r="B40" s="9">
         <v>1001</v>
       </c>
       <c r="C40" s="1">
@@ -1524,7 +3643,7 @@
       <c r="A41" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="9">
         <v>1009</v>
       </c>
       <c r="C41" s="1">
@@ -1538,7 +3657,7 @@
       <c r="A42" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="9">
         <v>1002</v>
       </c>
       <c r="C42" s="1">
@@ -1549,7 +3668,7 @@
       <c r="A43" t="s">
         <v>14</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="9">
         <v>1010</v>
       </c>
       <c r="C43" s="1">
@@ -1560,10 +3679,10 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B44" s="8">
+      <c r="B44" s="9">
         <v>1007</v>
       </c>
       <c r="C44" s="1">
@@ -1574,10 +3693,10 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="9">
         <v>1010</v>
       </c>
       <c r="C45" s="1">
@@ -1591,7 +3710,7 @@
       <c r="A46" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="9">
         <v>1007</v>
       </c>
       <c r="C46" s="1">
@@ -1698,7 +3817,7 @@
       <c r="F4" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -2033,7 +4152,7 @@
       <c r="D21" s="1">
         <v>45297</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="4">
         <v>74.02</v>
       </c>
       <c r="F21" t="s">
@@ -2353,14 +4472,14 @@
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
@@ -2374,7 +4493,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B2" t="s">
@@ -2388,7 +4507,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B3" t="s">
@@ -2402,7 +4521,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>27</v>
       </c>
       <c r="B4" t="s">
@@ -2416,7 +4535,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>19</v>
       </c>
       <c r="B5" t="s">
@@ -2430,7 +4549,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B6" t="s">
@@ -2444,7 +4563,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>23</v>
       </c>
       <c r="B7" t="s">
@@ -2458,7 +4577,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B8" t="s">
@@ -2472,7 +4591,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
@@ -2486,7 +4605,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B10" t="s">
@@ -2500,7 +4619,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B11" t="s">
@@ -2514,7 +4633,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B12" t="s">
@@ -2528,7 +4647,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B13" t="s">
@@ -2550,12 +4669,163 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B8FDEFF-4939-1C4F-8879-2780C4DDA6EF}">
+  <dimension ref="A3:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="11">
+        <v>7</v>
+      </c>
+      <c r="C5" s="11">
+        <v>3</v>
+      </c>
+      <c r="D5" s="11">
+        <v>2</v>
+      </c>
+      <c r="E5" s="11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="11">
+        <v>9</v>
+      </c>
+      <c r="C6" s="11">
+        <v>2</v>
+      </c>
+      <c r="D6" s="11">
+        <v>1</v>
+      </c>
+      <c r="E6" s="11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11">
+        <v>4</v>
+      </c>
+      <c r="D7" s="11">
+        <v>6</v>
+      </c>
+      <c r="E7" s="11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="11">
+        <v>2</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11">
+        <v>2</v>
+      </c>
+      <c r="E8" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11">
+        <v>4</v>
+      </c>
+      <c r="E9" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11">
+        <v>2</v>
+      </c>
+      <c r="D10" s="11">
+        <v>1</v>
+      </c>
+      <c r="E10" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="11">
+        <v>18</v>
+      </c>
+      <c r="C11" s="11">
+        <v>11</v>
+      </c>
+      <c r="D11" s="11">
+        <v>16</v>
+      </c>
+      <c r="E11" s="11">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{372024AA-7BEC-0A4F-ACDC-7D226F53D316}">
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" customWidth="1"/>
@@ -2572,7 +4842,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -2610,7 +4880,7 @@
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="9">
         <v>1009</v>
       </c>
       <c r="C2" s="1">
@@ -2636,15 +4906,15 @@
         <f>VLOOKUP(A2,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J2" s="10" t="str">
+      <c r="J2" s="11" t="str">
         <f>VLOOKUP(B2&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Univ.Prof. Heimo Karge</v>
       </c>
-      <c r="K2" s="10" t="str">
+      <c r="K2" s="11" t="str">
         <f>VLOOKUP(B2&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Marketing</v>
       </c>
-      <c r="L2" s="10" t="str">
+      <c r="L2" s="11" t="str">
         <f>VLOOKUP(B2&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -2653,7 +4923,7 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>1008</v>
       </c>
       <c r="C3" s="1">
@@ -2682,15 +4952,15 @@
         <f>VLOOKUP(A3,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J3" s="10" t="str">
+      <c r="J3" s="11" t="str">
         <f>VLOOKUP(B3&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Dipl.-Ing. Klaus-Werner Holsten B.Sc.</v>
       </c>
-      <c r="K3" s="10" t="str">
+      <c r="K3" s="11" t="str">
         <f>VLOOKUP(B3&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L3" s="10" t="str">
+      <c r="L3" s="11" t="str">
         <f>VLOOKUP(B3&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -2699,7 +4969,7 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>1005</v>
       </c>
       <c r="C4" s="1">
@@ -2728,15 +4998,15 @@
         <f>VLOOKUP(A4,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J4" s="10" t="str">
+      <c r="J4" s="11" t="str">
         <f>VLOOKUP(B4&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Alexandre Davids</v>
       </c>
-      <c r="K4" s="10" t="str">
+      <c r="K4" s="11" t="str">
         <f>VLOOKUP(B4&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L4" s="10" t="str">
+      <c r="L4" s="11" t="str">
         <f>VLOOKUP(B4&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -2745,7 +5015,7 @@
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <v>1010</v>
       </c>
       <c r="C5" s="1">
@@ -2771,15 +5041,15 @@
         <f>VLOOKUP(A5,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J5" s="10" t="str">
+      <c r="J5" s="11" t="str">
         <f>VLOOKUP(B5&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Carolin Hande</v>
       </c>
-      <c r="K5" s="10" t="str">
+      <c r="K5" s="11" t="str">
         <f>VLOOKUP(B5&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L5" s="10" t="str">
+      <c r="L5" s="11" t="str">
         <f>VLOOKUP(B5&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -2788,7 +5058,7 @@
       <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>1012</v>
       </c>
       <c r="C6" s="1">
@@ -2817,15 +5087,15 @@
         <f>VLOOKUP(A6,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J6" s="10" t="str">
+      <c r="J6" s="11" t="str">
         <f>VLOOKUP(B6&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Ariane Klemt-Kaul</v>
       </c>
-      <c r="K6" s="10" t="str">
+      <c r="K6" s="11" t="str">
         <f>VLOOKUP(B6&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L6" s="10" t="str">
+      <c r="L6" s="11" t="str">
         <f>VLOOKUP(B6&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>München</v>
       </c>
@@ -2834,7 +5104,7 @@
       <c r="A7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <v>1009</v>
       </c>
       <c r="C7" s="1">
@@ -2860,24 +5130,24 @@
         <f>VLOOKUP(A7,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J7" s="10" t="str">
+      <c r="J7" s="11" t="str">
         <f>VLOOKUP(B7&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Univ.Prof. Heimo Karge</v>
       </c>
-      <c r="K7" s="10" t="str">
+      <c r="K7" s="11" t="str">
         <f>VLOOKUP(B7&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Marketing</v>
       </c>
-      <c r="L7" s="10" t="str">
+      <c r="L7" s="11" t="str">
         <f>VLOOKUP(B7&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="9">
         <v>1011</v>
       </c>
       <c r="C8" s="1">
@@ -2906,15 +5176,15 @@
         <f>VLOOKUP(A8,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J8" s="10" t="str">
+      <c r="J8" s="11" t="str">
         <f>VLOOKUP(B8&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Auguste Davids</v>
       </c>
-      <c r="K8" s="10" t="str">
+      <c r="K8" s="11" t="str">
         <f>VLOOKUP(B8&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L8" s="10" t="str">
+      <c r="L8" s="11" t="str">
         <f>VLOOKUP(B8&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -2923,7 +5193,7 @@
       <c r="A9" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="9">
         <v>1005</v>
       </c>
       <c r="C9" s="1">
@@ -2952,15 +5222,15 @@
         <f>VLOOKUP(A9,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J9" s="10" t="str">
+      <c r="J9" s="11" t="str">
         <f>VLOOKUP(B9&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Alexandre Davids</v>
       </c>
-      <c r="K9" s="10" t="str">
+      <c r="K9" s="11" t="str">
         <f>VLOOKUP(B9&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L9" s="10" t="str">
+      <c r="L9" s="11" t="str">
         <f>VLOOKUP(B9&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -2969,7 +5239,7 @@
       <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <v>1004</v>
       </c>
       <c r="C10" s="1">
@@ -2995,15 +5265,15 @@
         <f>VLOOKUP(A10,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J10" s="10" t="str">
+      <c r="J10" s="11" t="str">
         <f>VLOOKUP(B10&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Klemens Löffler</v>
       </c>
-      <c r="K10" s="10" t="str">
+      <c r="K10" s="11" t="str">
         <f>VLOOKUP(B10&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L10" s="10" t="str">
+      <c r="L10" s="11" t="str">
         <f>VLOOKUP(B10&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3012,7 +5282,7 @@
       <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <v>1012</v>
       </c>
       <c r="C11" s="1">
@@ -3041,15 +5311,15 @@
         <f>VLOOKUP(A11,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J11" s="10" t="str">
+      <c r="J11" s="11" t="str">
         <f>VLOOKUP(B11&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Ariane Klemt-Kaul</v>
       </c>
-      <c r="K11" s="10" t="str">
+      <c r="K11" s="11" t="str">
         <f>VLOOKUP(B11&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L11" s="10" t="str">
+      <c r="L11" s="11" t="str">
         <f>VLOOKUP(B11&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>München</v>
       </c>
@@ -3058,7 +5328,7 @@
       <c r="A12" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <v>1008</v>
       </c>
       <c r="C12" s="1">
@@ -3084,15 +5354,15 @@
         <f>VLOOKUP(A12,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J12" s="10" t="str">
+      <c r="J12" s="11" t="str">
         <f>VLOOKUP(B12&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Dipl.-Ing. Klaus-Werner Holsten B.Sc.</v>
       </c>
-      <c r="K12" s="10" t="str">
+      <c r="K12" s="11" t="str">
         <f>VLOOKUP(B12&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L12" s="10" t="str">
+      <c r="L12" s="11" t="str">
         <f>VLOOKUP(B12&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3101,7 +5371,7 @@
       <c r="A13" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>1002</v>
       </c>
       <c r="C13" s="1">
@@ -3130,15 +5400,15 @@
         <f>VLOOKUP(A13,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J13" s="10" t="str">
+      <c r="J13" s="11" t="str">
         <f>VLOOKUP(B13&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eleni Hauffer</v>
       </c>
-      <c r="K13" s="10" t="str">
+      <c r="K13" s="11" t="str">
         <f>VLOOKUP(B13&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L13" s="10" t="str">
+      <c r="L13" s="11" t="str">
         <f>VLOOKUP(B13&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3147,7 +5417,7 @@
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>1006</v>
       </c>
       <c r="C14" s="1">
@@ -3176,15 +5446,15 @@
         <f>VLOOKUP(A14,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J14" s="10" t="str">
+      <c r="J14" s="11" t="str">
         <f>VLOOKUP(B14&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eric Patberg B.Sc.</v>
       </c>
-      <c r="K14" s="10" t="str">
+      <c r="K14" s="11" t="str">
         <f>VLOOKUP(B14&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L14" s="10" t="str">
+      <c r="L14" s="11" t="str">
         <f>VLOOKUP(B14&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3193,7 +5463,7 @@
       <c r="A15" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="9">
         <v>1010</v>
       </c>
       <c r="C15" s="1">
@@ -3206,7 +5476,7 @@
         <f>VLOOKUP(A15,Geraete!A:F,2,FALSE)</f>
         <v>Smartphone</v>
       </c>
-      <c r="F15" s="4" t="str">
+      <c r="F15" s="5" t="str">
         <f>VLOOKUP(A15,Geraete!A:F,3,FALSE)</f>
         <v>iPhone 13</v>
       </c>
@@ -3222,15 +5492,15 @@
         <f>VLOOKUP(A15,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J15" s="10" t="str">
+      <c r="J15" s="11" t="str">
         <f>VLOOKUP(B15&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Carolin Hande</v>
       </c>
-      <c r="K15" s="10" t="str">
+      <c r="K15" s="11" t="str">
         <f>VLOOKUP(B15&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L15" s="10" t="str">
+      <c r="L15" s="11" t="str">
         <f>VLOOKUP(B15&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3239,7 +5509,7 @@
       <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="9">
         <v>1012</v>
       </c>
       <c r="C16" s="1">
@@ -3265,15 +5535,15 @@
         <f>VLOOKUP(A16,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J16" s="10" t="str">
+      <c r="J16" s="11" t="str">
         <f>VLOOKUP(B16&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Ariane Klemt-Kaul</v>
       </c>
-      <c r="K16" s="10" t="str">
+      <c r="K16" s="11" t="str">
         <f>VLOOKUP(B16&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L16" s="10" t="str">
+      <c r="L16" s="11" t="str">
         <f>VLOOKUP(B16&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>München</v>
       </c>
@@ -3282,7 +5552,7 @@
       <c r="A17" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="9">
         <v>1002</v>
       </c>
       <c r="C17" s="1">
@@ -3308,15 +5578,15 @@
         <f>VLOOKUP(A17,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J17" s="10" t="str">
+      <c r="J17" s="11" t="str">
         <f>VLOOKUP(B17&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eleni Hauffer</v>
       </c>
-      <c r="K17" s="10" t="str">
+      <c r="K17" s="11" t="str">
         <f>VLOOKUP(B17&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L17" s="10" t="str">
+      <c r="L17" s="11" t="str">
         <f>VLOOKUP(B17&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3325,7 +5595,7 @@
       <c r="A18" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>1002</v>
       </c>
       <c r="C18" s="1">
@@ -3354,15 +5624,15 @@
         <f>VLOOKUP(A18,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J18" s="10" t="str">
+      <c r="J18" s="11" t="str">
         <f>VLOOKUP(B18&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eleni Hauffer</v>
       </c>
-      <c r="K18" s="10" t="str">
+      <c r="K18" s="11" t="str">
         <f>VLOOKUP(B18&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L18" s="10" t="str">
+      <c r="L18" s="11" t="str">
         <f>VLOOKUP(B18&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3371,7 +5641,7 @@
       <c r="A19" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>1011</v>
       </c>
       <c r="C19" s="1">
@@ -3400,15 +5670,15 @@
         <f>VLOOKUP(A19,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J19" s="10" t="str">
+      <c r="J19" s="11" t="str">
         <f>VLOOKUP(B19&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Auguste Davids</v>
       </c>
-      <c r="K19" s="10" t="str">
+      <c r="K19" s="11" t="str">
         <f>VLOOKUP(B19&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L19" s="10" t="str">
+      <c r="L19" s="11" t="str">
         <f>VLOOKUP(B19&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3417,7 +5687,7 @@
       <c r="A20" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>1003</v>
       </c>
       <c r="C20" s="1">
@@ -3443,24 +5713,24 @@
         <f>VLOOKUP(A20,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J20" s="10" t="str">
+      <c r="J20" s="11" t="str">
         <f>VLOOKUP(B20&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Paul Dobes-Stiffel</v>
       </c>
-      <c r="K20" s="10" t="str">
+      <c r="K20" s="11" t="str">
         <f>VLOOKUP(B20&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Produktion</v>
       </c>
-      <c r="L20" s="10" t="str">
+      <c r="L20" s="11" t="str">
         <f>VLOOKUP(B20&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="A21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="9">
         <v>1004</v>
       </c>
       <c r="C21" s="1">
@@ -3486,15 +5756,15 @@
         <f>VLOOKUP(A21,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J21" s="10" t="str">
+      <c r="J21" s="11" t="str">
         <f>VLOOKUP(B21&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Klemens Löffler</v>
       </c>
-      <c r="K21" s="10" t="str">
+      <c r="K21" s="11" t="str">
         <f>VLOOKUP(B21&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L21" s="10" t="str">
+      <c r="L21" s="11" t="str">
         <f>VLOOKUP(B21&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3503,7 +5773,7 @@
       <c r="A22" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="9">
         <v>1004</v>
       </c>
       <c r="C22" s="1">
@@ -3532,15 +5802,15 @@
         <f>VLOOKUP(A22,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J22" s="10" t="str">
+      <c r="J22" s="11" t="str">
         <f>VLOOKUP(B22&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Klemens Löffler</v>
       </c>
-      <c r="K22" s="10" t="str">
+      <c r="K22" s="11" t="str">
         <f>VLOOKUP(B22&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L22" s="10" t="str">
+      <c r="L22" s="11" t="str">
         <f>VLOOKUP(B22&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3549,7 +5819,7 @@
       <c r="A23" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="9">
         <v>1006</v>
       </c>
       <c r="C23" s="1">
@@ -3578,15 +5848,15 @@
         <f>VLOOKUP(A23,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J23" s="10" t="str">
+      <c r="J23" s="11" t="str">
         <f>VLOOKUP(B23&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eric Patberg B.Sc.</v>
       </c>
-      <c r="K23" s="10" t="str">
+      <c r="K23" s="11" t="str">
         <f>VLOOKUP(B23&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L23" s="10" t="str">
+      <c r="L23" s="11" t="str">
         <f>VLOOKUP(B23&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3595,7 +5865,7 @@
       <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="9">
         <v>1012</v>
       </c>
       <c r="C24" s="1">
@@ -3624,15 +5894,15 @@
         <f>VLOOKUP(A24,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J24" s="10" t="str">
+      <c r="J24" s="11" t="str">
         <f>VLOOKUP(B24&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Ariane Klemt-Kaul</v>
       </c>
-      <c r="K24" s="10" t="str">
+      <c r="K24" s="11" t="str">
         <f>VLOOKUP(B24&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L24" s="10" t="str">
+      <c r="L24" s="11" t="str">
         <f>VLOOKUP(B24&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>München</v>
       </c>
@@ -3641,7 +5911,7 @@
       <c r="A25" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="9">
         <v>1001</v>
       </c>
       <c r="C25" s="1">
@@ -3670,15 +5940,15 @@
         <f>VLOOKUP(A25,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J25" s="10" t="str">
+      <c r="J25" s="11" t="str">
         <f>VLOOKUP(B25&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Aleksandr Weinhage</v>
       </c>
-      <c r="K25" s="10" t="str">
+      <c r="K25" s="11" t="str">
         <f>VLOOKUP(B25&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L25" s="10" t="str">
+      <c r="L25" s="11" t="str">
         <f>VLOOKUP(B25&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3687,7 +5957,7 @@
       <c r="A26" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>1002</v>
       </c>
       <c r="C26" s="1">
@@ -3716,15 +5986,15 @@
         <f>VLOOKUP(A26,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J26" s="10" t="str">
+      <c r="J26" s="11" t="str">
         <f>VLOOKUP(B26&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eleni Hauffer</v>
       </c>
-      <c r="K26" s="10" t="str">
+      <c r="K26" s="11" t="str">
         <f>VLOOKUP(B26&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L26" s="10" t="str">
+      <c r="L26" s="11" t="str">
         <f>VLOOKUP(B26&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3733,7 +6003,7 @@
       <c r="A27" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>1009</v>
       </c>
       <c r="C27" s="1">
@@ -3762,15 +6032,15 @@
         <f>VLOOKUP(A27,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J27" s="10" t="str">
+      <c r="J27" s="11" t="str">
         <f>VLOOKUP(B27&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Univ.Prof. Heimo Karge</v>
       </c>
-      <c r="K27" s="10" t="str">
+      <c r="K27" s="11" t="str">
         <f>VLOOKUP(B27&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Marketing</v>
       </c>
-      <c r="L27" s="10" t="str">
+      <c r="L27" s="11" t="str">
         <f>VLOOKUP(B27&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -3779,7 +6049,7 @@
       <c r="A28" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="9">
         <v>1003</v>
       </c>
       <c r="C28" s="1">
@@ -3808,24 +6078,24 @@
         <f>VLOOKUP(A28,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J28" s="10" t="str">
+      <c r="J28" s="11" t="str">
         <f>VLOOKUP(B28&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Paul Dobes-Stiffel</v>
       </c>
-      <c r="K28" s="10" t="str">
+      <c r="K28" s="11" t="str">
         <f>VLOOKUP(B28&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Produktion</v>
       </c>
-      <c r="L28" s="10" t="str">
+      <c r="L28" s="11" t="str">
         <f>VLOOKUP(B28&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>1002</v>
       </c>
       <c r="C29" s="1">
@@ -3854,15 +6124,15 @@
         <f>VLOOKUP(A29,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J29" s="10" t="str">
+      <c r="J29" s="11" t="str">
         <f>VLOOKUP(B29&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eleni Hauffer</v>
       </c>
-      <c r="K29" s="10" t="str">
+      <c r="K29" s="11" t="str">
         <f>VLOOKUP(B29&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L29" s="10" t="str">
+      <c r="L29" s="11" t="str">
         <f>VLOOKUP(B29&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3871,7 +6141,7 @@
       <c r="A30" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="9">
         <v>1001</v>
       </c>
       <c r="C30" s="1">
@@ -3897,15 +6167,15 @@
         <f>VLOOKUP(A30,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J30" s="10" t="str">
+      <c r="J30" s="11" t="str">
         <f>VLOOKUP(B30&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Aleksandr Weinhage</v>
       </c>
-      <c r="K30" s="10" t="str">
+      <c r="K30" s="11" t="str">
         <f>VLOOKUP(B30&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L30" s="10" t="str">
+      <c r="L30" s="11" t="str">
         <f>VLOOKUP(B30&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -3914,7 +6184,7 @@
       <c r="A31" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="9">
         <v>1001</v>
       </c>
       <c r="C31" s="1">
@@ -3940,24 +6210,24 @@
         <f>VLOOKUP(A31,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J31" s="10" t="str">
+      <c r="J31" s="11" t="str">
         <f>VLOOKUP(B31&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Aleksandr Weinhage</v>
       </c>
-      <c r="K31" s="10" t="str">
+      <c r="K31" s="11" t="str">
         <f>VLOOKUP(B31&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L31" s="10" t="str">
+      <c r="L31" s="11" t="str">
         <f>VLOOKUP(B31&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="9">
         <v>1003</v>
       </c>
       <c r="C32" s="1">
@@ -3986,24 +6256,24 @@
         <f>VLOOKUP(A32,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J32" s="10" t="str">
+      <c r="J32" s="11" t="str">
         <f>VLOOKUP(B32&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Paul Dobes-Stiffel</v>
       </c>
-      <c r="K32" s="10" t="str">
+      <c r="K32" s="11" t="str">
         <f>VLOOKUP(B32&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Produktion</v>
       </c>
-      <c r="L32" s="10" t="str">
+      <c r="L32" s="11" t="str">
         <f>VLOOKUP(B32&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="A33" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="9">
         <v>1004</v>
       </c>
       <c r="C33" s="1">
@@ -4029,24 +6299,24 @@
         <f>VLOOKUP(A33,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J33" s="10" t="str">
+      <c r="J33" s="11" t="str">
         <f>VLOOKUP(B33&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Klemens Löffler</v>
       </c>
-      <c r="K33" s="10" t="str">
+      <c r="K33" s="11" t="str">
         <f>VLOOKUP(B33&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L33" s="10" t="str">
+      <c r="L33" s="11" t="str">
         <f>VLOOKUP(B33&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="9">
         <v>1003</v>
       </c>
       <c r="C34" s="1">
@@ -4075,15 +6345,15 @@
         <f>VLOOKUP(A34,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J34" s="10" t="str">
+      <c r="J34" s="11" t="str">
         <f>VLOOKUP(B34&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Paul Dobes-Stiffel</v>
       </c>
-      <c r="K34" s="10" t="str">
+      <c r="K34" s="11" t="str">
         <f>VLOOKUP(B34&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Produktion</v>
       </c>
-      <c r="L34" s="10" t="str">
+      <c r="L34" s="11" t="str">
         <f>VLOOKUP(B34&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -4092,7 +6362,7 @@
       <c r="A35" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="9">
         <v>1005</v>
       </c>
       <c r="C35" s="1">
@@ -4118,15 +6388,15 @@
         <f>VLOOKUP(A35,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J35" s="10" t="str">
+      <c r="J35" s="11" t="str">
         <f>VLOOKUP(B35&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Alexandre Davids</v>
       </c>
-      <c r="K35" s="10" t="str">
+      <c r="K35" s="11" t="str">
         <f>VLOOKUP(B35&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L35" s="10" t="str">
+      <c r="L35" s="11" t="str">
         <f>VLOOKUP(B35&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -4135,7 +6405,7 @@
       <c r="A36" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="9">
         <v>1005</v>
       </c>
       <c r="C36" s="1">
@@ -4164,15 +6434,15 @@
         <f>VLOOKUP(A36,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J36" s="10" t="str">
+      <c r="J36" s="11" t="str">
         <f>VLOOKUP(B36&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Alexandre Davids</v>
       </c>
-      <c r="K36" s="10" t="str">
+      <c r="K36" s="11" t="str">
         <f>VLOOKUP(B36&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Vertrieb</v>
       </c>
-      <c r="L36" s="10" t="str">
+      <c r="L36" s="11" t="str">
         <f>VLOOKUP(B36&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -4181,7 +6451,7 @@
       <c r="A37" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>1003</v>
       </c>
       <c r="C37" s="1">
@@ -4210,15 +6480,15 @@
         <f>VLOOKUP(A37,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J37" s="10" t="str">
+      <c r="J37" s="11" t="str">
         <f>VLOOKUP(B37&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Paul Dobes-Stiffel</v>
       </c>
-      <c r="K37" s="10" t="str">
+      <c r="K37" s="11" t="str">
         <f>VLOOKUP(B37&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Produktion</v>
       </c>
-      <c r="L37" s="10" t="str">
+      <c r="L37" s="11" t="str">
         <f>VLOOKUP(B37&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -4227,7 +6497,7 @@
       <c r="A38" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>1001</v>
       </c>
       <c r="C38" s="1">
@@ -4256,15 +6526,15 @@
         <f>VLOOKUP(A38,Geraete!A:F,6,FALSE)</f>
         <v>Hamburg</v>
       </c>
-      <c r="J38" s="10" t="str">
+      <c r="J38" s="11" t="str">
         <f>VLOOKUP(B38&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Aleksandr Weinhage</v>
       </c>
-      <c r="K38" s="10" t="str">
+      <c r="K38" s="11" t="str">
         <f>VLOOKUP(B38&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L38" s="10" t="str">
+      <c r="L38" s="11" t="str">
         <f>VLOOKUP(B38&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -4273,7 +6543,7 @@
       <c r="A39" t="s">
         <v>4</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="9">
         <v>1001</v>
       </c>
       <c r="C39" s="1">
@@ -4299,24 +6569,24 @@
         <f>VLOOKUP(A39,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J39" s="10" t="str">
+      <c r="J39" s="11" t="str">
         <f>VLOOKUP(B39&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Aleksandr Weinhage</v>
       </c>
-      <c r="K39" s="10" t="str">
+      <c r="K39" s="11" t="str">
         <f>VLOOKUP(B39&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L39" s="10" t="str">
+      <c r="L39" s="11" t="str">
         <f>VLOOKUP(B39&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B40" s="8">
+      <c r="B40" s="9">
         <v>1001</v>
       </c>
       <c r="C40" s="1">
@@ -4345,15 +6615,15 @@
         <f>VLOOKUP(A40,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J40" s="10" t="str">
+      <c r="J40" s="11" t="str">
         <f>VLOOKUP(B40&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Aleksandr Weinhage</v>
       </c>
-      <c r="K40" s="10" t="str">
+      <c r="K40" s="11" t="str">
         <f>VLOOKUP(B40&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L40" s="10" t="str">
+      <c r="L40" s="11" t="str">
         <f>VLOOKUP(B40&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -4362,7 +6632,7 @@
       <c r="A41" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="9">
         <v>1009</v>
       </c>
       <c r="C41" s="1">
@@ -4391,15 +6661,15 @@
         <f>VLOOKUP(A41,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J41" s="10" t="str">
+      <c r="J41" s="11" t="str">
         <f>VLOOKUP(B41&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Univ.Prof. Heimo Karge</v>
       </c>
-      <c r="K41" s="10" t="str">
+      <c r="K41" s="11" t="str">
         <f>VLOOKUP(B41&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>Marketing</v>
       </c>
-      <c r="L41" s="10" t="str">
+      <c r="L41" s="11" t="str">
         <f>VLOOKUP(B41&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -4408,7 +6678,7 @@
       <c r="A42" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="9">
         <v>1002</v>
       </c>
       <c r="C42" s="1">
@@ -4434,15 +6704,15 @@
         <f>VLOOKUP(A42,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J42" s="10" t="str">
+      <c r="J42" s="11" t="str">
         <f>VLOOKUP(B42&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Eleni Hauffer</v>
       </c>
-      <c r="K42" s="10" t="str">
+      <c r="K42" s="11" t="str">
         <f>VLOOKUP(B42&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L42" s="10" t="str">
+      <c r="L42" s="11" t="str">
         <f>VLOOKUP(B42&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
@@ -4451,7 +6721,7 @@
       <c r="A43" t="s">
         <v>14</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="9">
         <v>1010</v>
       </c>
       <c r="C43" s="1">
@@ -4480,24 +6750,24 @@
         <f>VLOOKUP(A43,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J43" s="10" t="str">
+      <c r="J43" s="11" t="str">
         <f>VLOOKUP(B43&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Carolin Hande</v>
       </c>
-      <c r="K43" s="10" t="str">
+      <c r="K43" s="11" t="str">
         <f>VLOOKUP(B43&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L43" s="10" t="str">
+      <c r="L43" s="11" t="str">
         <f>VLOOKUP(B43&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B44" s="8">
+      <c r="B44" s="9">
         <v>1007</v>
       </c>
       <c r="C44" s="1">
@@ -4526,24 +6796,24 @@
         <f>VLOOKUP(A44,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J44" s="10" t="str">
+      <c r="J44" s="11" t="str">
         <f>VLOOKUP(B44&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Orhan Siering MBA.</v>
       </c>
-      <c r="K44" s="10" t="str">
+      <c r="K44" s="11" t="str">
         <f>VLOOKUP(B44&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L44" s="10" t="str">
+      <c r="L44" s="11" t="str">
         <f>VLOOKUP(B44&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="9">
         <v>1010</v>
       </c>
       <c r="C45" s="1">
@@ -4572,15 +6842,15 @@
         <f>VLOOKUP(A45,Geraete!A:F,6,FALSE)</f>
         <v>Berlin</v>
       </c>
-      <c r="J45" s="10" t="str">
+      <c r="J45" s="11" t="str">
         <f>VLOOKUP(B45&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Carolin Hande</v>
       </c>
-      <c r="K45" s="10" t="str">
+      <c r="K45" s="11" t="str">
         <f>VLOOKUP(B45&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L45" s="10" t="str">
+      <c r="L45" s="11" t="str">
         <f>VLOOKUP(B45&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Hamburg</v>
       </c>
@@ -4589,7 +6859,7 @@
       <c r="A46" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="9">
         <v>1007</v>
       </c>
       <c r="C46" s="1">
@@ -4615,18 +6885,27 @@
         <f>VLOOKUP(A46,Geraete!A:F,6,FALSE)</f>
         <v>München</v>
       </c>
-      <c r="J46" s="10" t="str">
+      <c r="J46" s="11" t="str">
         <f>VLOOKUP(B46&amp;"",Mitarbeiter!$A:$D,2,FALSE)</f>
         <v>Orhan Siering MBA.</v>
       </c>
-      <c r="K46" s="10" t="str">
+      <c r="K46" s="11" t="str">
         <f>VLOOKUP(B46&amp;"",Mitarbeiter!$A:$D,3,FALSE)</f>
         <v>IT</v>
       </c>
-      <c r="L46" s="10" t="str">
+      <c r="L46" s="11" t="str">
         <f>VLOOKUP(B46&amp;"",Mitarbeiter!$A:$D,4,FALSE)</f>
         <v>Berlin</v>
       </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="11"/>
+      <c r="I47" s="11"/>
+      <c r="J47" s="11"/>
+      <c r="K47" s="11"/>
+      <c r="L47" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>